<commit_message>
tambah menu data aids
</commit_message>
<xml_diff>
--- a/excel/contoh_tbc.xlsx
+++ b/excel/contoh_tbc.xlsx
@@ -1,17 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="6" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\satset\wp-content\plugins\wp-satset\excel\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2DAEE4B-16B7-498B-9F27-6479113EEBCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="8235"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="124519"/>
-  <extLst xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -24,9 +30,6 @@
     <t>0005</t>
   </si>
   <si>
-    <t>3520.1622</t>
-  </si>
-  <si>
     <t>P</t>
   </si>
   <si>
@@ -39,27 +42,18 @@
     <t>0006</t>
   </si>
   <si>
-    <t>3520.1621</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
     <t>0023</t>
   </si>
   <si>
-    <t>3520.1618</t>
-  </si>
-  <si>
     <t>L</t>
   </si>
   <si>
     <t>0004</t>
   </si>
   <si>
-    <t>3520.1616</t>
-  </si>
-  <si>
     <t>no</t>
   </si>
   <si>
@@ -121,13 +115,25 @@
   </si>
   <si>
     <t>Jl. D , Suratmajan, Kec. Maospati, Kab. Magetan, Jawa Timur</t>
+  </si>
+  <si>
+    <t>desa</t>
+  </si>
+  <si>
+    <t>kecamatan</t>
+  </si>
+  <si>
+    <t>kabkot</t>
+  </si>
+  <si>
+    <t>provinsi</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -444,16 +450,16 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:S5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.5703125" bestFit="1" customWidth="1"/>
@@ -462,61 +468,77 @@
     <col min="6" max="6" width="45.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="43.5703125" customWidth="1"/>
-    <col min="10" max="10" width="31.7109375" customWidth="1"/>
-    <col min="11" max="11" width="30.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="30.140625" customWidth="1"/>
-    <col min="14" max="14" width="19" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.85546875" customWidth="1"/>
+    <col min="11" max="11" width="16.42578125" customWidth="1"/>
+    <col min="12" max="12" width="17.42578125" customWidth="1"/>
+    <col min="13" max="13" width="16.42578125" customWidth="1"/>
+    <col min="14" max="14" width="31.7109375" customWidth="1"/>
+    <col min="15" max="15" width="30.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="30.140625" customWidth="1"/>
+    <col min="18" max="18" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="J1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>27</v>
-      </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -526,35 +548,35 @@
       <c r="C2" t="s">
         <v>0</v>
       </c>
-      <c r="D2" t="s">
-        <v>1</v>
+      <c r="D2">
+        <v>35201622</v>
       </c>
       <c r="E2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G2">
         <v>53</v>
       </c>
       <c r="H2" t="s">
+        <v>1</v>
+      </c>
+      <c r="I2" t="s">
+        <v>26</v>
+      </c>
+      <c r="O2" t="s">
         <v>2</v>
       </c>
-      <c r="I2" t="s">
-        <v>30</v>
-      </c>
-      <c r="K2" t="s">
+      <c r="P2" s="2">
+        <v>44960.0000462963</v>
+      </c>
+      <c r="R2" t="s">
         <v>3</v>
       </c>
-      <c r="L2" s="2">
-        <v>44960.0000462963</v>
-      </c>
-      <c r="N2" t="s">
-        <v>4</v>
-      </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -562,40 +584,40 @@
         <v>44960.0000462963</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" t="s">
-        <v>6</v>
+        <v>4</v>
+      </c>
+      <c r="D3">
+        <v>35201621</v>
       </c>
       <c r="E3" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F3" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G3">
         <v>57</v>
       </c>
       <c r="H3" t="s">
+        <v>1</v>
+      </c>
+      <c r="I3" t="s">
+        <v>27</v>
+      </c>
+      <c r="O3" t="s">
         <v>2</v>
       </c>
-      <c r="I3" t="s">
-        <v>31</v>
-      </c>
-      <c r="K3" t="s">
+      <c r="P3" s="2">
+        <v>44960.0000462963</v>
+      </c>
+      <c r="R3" t="s">
         <v>3</v>
       </c>
-      <c r="L3" s="2">
-        <v>44960.0000462963</v>
-      </c>
-      <c r="N3" t="s">
-        <v>4</v>
-      </c>
-      <c r="O3" t="s">
-        <v>7</v>
+      <c r="S3" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -603,37 +625,37 @@
         <v>44959.0000462963</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" t="s">
-        <v>9</v>
+        <v>6</v>
+      </c>
+      <c r="D4">
+        <v>35201618</v>
       </c>
       <c r="E4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F4" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G4">
         <v>6</v>
       </c>
       <c r="H4" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="I4" t="s">
-        <v>32</v>
-      </c>
-      <c r="K4" t="s">
+        <v>28</v>
+      </c>
+      <c r="O4" t="s">
+        <v>2</v>
+      </c>
+      <c r="P4" s="2">
+        <v>44959.0000462963</v>
+      </c>
+      <c r="R4" t="s">
         <v>3</v>
       </c>
-      <c r="L4" s="2">
-        <v>44959.0000462963</v>
-      </c>
-      <c r="N4" t="s">
-        <v>4</v>
-      </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2</v>
       </c>
@@ -641,34 +663,34 @@
         <v>44958.0000462963</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" t="s">
-        <v>12</v>
+        <v>8</v>
+      </c>
+      <c r="D5">
+        <v>35201616</v>
       </c>
       <c r="E5" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F5" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G5">
         <v>65</v>
       </c>
       <c r="H5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="I5" t="s">
-        <v>33</v>
-      </c>
-      <c r="K5" t="s">
+        <v>29</v>
+      </c>
+      <c r="O5" t="s">
+        <v>2</v>
+      </c>
+      <c r="P5" s="2">
+        <v>44958.0000462963</v>
+      </c>
+      <c r="R5" t="s">
         <v>3</v>
-      </c>
-      <c r="L5" s="2">
-        <v>44958.0000462963</v>
-      </c>
-      <c r="N5" t="s">
-        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>